<commit_message>
📊 Actualización automática del dashboard
</commit_message>
<xml_diff>
--- a/Comentarios Campaña.xlsx
+++ b/Comentarios Campaña.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P134"/>
+  <dimension ref="A1:P138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8220,6 +8220,174 @@
         </is>
       </c>
       <c r="P134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>15</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DU1R9xFAP4q/</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DU1R9xFAP4q/</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr"/>
+      <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr"/>
+      <c r="H135" t="inlineStr"/>
+      <c r="I135" t="inlineStr"/>
+      <c r="J135" t="inlineStr"/>
+      <c r="K135" t="n">
+        <v>0</v>
+      </c>
+      <c r="L135" t="n">
+        <v>0</v>
+      </c>
+      <c r="M135" t="b">
+        <v>0</v>
+      </c>
+      <c r="N135" t="inlineStr"/>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>16</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DU1SXxMgAEP/</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DU1SXxMgAEP/</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr"/>
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr"/>
+      <c r="H136" t="inlineStr"/>
+      <c r="I136" t="inlineStr"/>
+      <c r="J136" t="inlineStr"/>
+      <c r="K136" t="n">
+        <v>0</v>
+      </c>
+      <c r="L136" t="n">
+        <v>0</v>
+      </c>
+      <c r="M136" t="b">
+        <v>0</v>
+      </c>
+      <c r="N136" t="inlineStr"/>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>17</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/100064867445065/posts/1352095373629365/</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/100064867445065/posts/1352095373629365/</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr"/>
+      <c r="H137" t="inlineStr"/>
+      <c r="I137" t="inlineStr"/>
+      <c r="J137" t="inlineStr"/>
+      <c r="K137" t="n">
+        <v>0</v>
+      </c>
+      <c r="L137" t="n">
+        <v>0</v>
+      </c>
+      <c r="M137" t="b">
+        <v>0</v>
+      </c>
+      <c r="N137" t="inlineStr"/>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>18</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/100064867445065/posts/1352097876962448/</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/100064867445065/posts/1352097876962448/</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr"/>
+      <c r="H138" t="inlineStr"/>
+      <c r="I138" t="inlineStr"/>
+      <c r="J138" t="inlineStr"/>
+      <c r="K138" t="n">
+        <v>0</v>
+      </c>
+      <c r="L138" t="n">
+        <v>0</v>
+      </c>
+      <c r="M138" t="b">
+        <v>0</v>
+      </c>
+      <c r="N138" t="inlineStr"/>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8232,7 +8400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8609,6 +8777,98 @@
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DU1R9xFAP4q/</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DU1SXxMgAEP/</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/100064867445065/posts/1352095373629365/</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Facebook</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/100064867445065/posts/1352097876962448/</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8719,7 +8979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8737,7 +8997,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUivrpRgMcb/</t>
+          <t>https://www.instagram.com/p/DU1R9xFAP4q/</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -8749,7 +9009,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUi6YciAMYK/</t>
+          <t>https://www.instagram.com/p/DU1SXxMgAEP/</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -8761,7 +9021,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUtaoL5APcG/</t>
+          <t>https://www.instagram.com/p/DUivrpRgMcb/</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8773,7 +9033,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUtakQ_ABbk/</t>
+          <t>https://www.instagram.com/p/DUi6YciAMYK/</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -8785,7 +9045,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUtaoIzAPIq/</t>
+          <t>https://www.instagram.com/p/DUtaoL5APcG/</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -8797,7 +9057,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/p/DUtalE5gKDU/</t>
+          <t>https://www.instagram.com/p/DUtakQ_ABbk/</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -8809,7 +9069,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/100064867445065/posts/1349346550570914/</t>
+          <t>https://www.instagram.com/p/DUtaoIzAPIq/</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -8821,7 +9081,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/100064867445065/posts/1349346470570922/</t>
+          <t>https://www.instagram.com/p/DUtalE5gKDU/</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8833,7 +9093,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/100064867445065/posts/1349346567237579/</t>
+          <t>https://www.facebook.com/100064867445065/posts/1349346550570914/</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -8845,10 +9105,58 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>https://www.facebook.com/100064867445065/posts/1349346470570922/</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>FAILED_ALL_ATTEMPTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/100064867445065/posts/1349346567237579/</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>FAILED_ALL_ATTEMPTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>https://www.facebook.com/100064867445065/posts/1349346463904256/</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>FAILED_ALL_ATTEMPTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/100064867445065/posts/1352095373629365/</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>FAILED_ALL_ATTEMPTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/100064867445065/posts/1352097876962448/</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
         <is>
           <t>FAILED_ALL_ATTEMPTS</t>
         </is>
@@ -8897,19 +9205,19 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B2" t="n">
         <v>4</v>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>33</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>